<commit_message>
Enhance FHIR XML processing with validation, date handling, and tests (#112)
</commit_message>
<xml_diff>
--- a/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
+++ b/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
@@ -1066,7 +1066,7 @@
         <v>39</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>31292</v>
+        <v>31293</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>14</v>
@@ -1573,7 +1573,7 @@
         <v>77</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>33010</v>
+        <v>33011</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>14</v>
@@ -1684,7 +1684,7 @@
         <v>85</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>30783</v>
+        <v>30784</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>14</v>
@@ -1719,7 +1719,7 @@
         <v>88</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>31606</v>
+        <v>31607</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>14</v>
@@ -1754,7 +1754,7 @@
         <v>30</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>29453</v>
+        <v>29452</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>89</v>
@@ -1827,7 +1827,7 @@
         <v>95</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>36386</v>
+        <v>36387</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>14</v>
@@ -2046,7 +2046,7 @@
         <v>69</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>32275</v>
+        <v>32274</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>89</v>

</xml_diff>

<commit_message>
Add patient that died in eg. excel file
</commit_message>
<xml_diff>
--- a/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
+++ b/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
@@ -11,7 +11,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$39</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$40</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="114">
   <si>
     <t xml:space="preserve">patient_ref</t>
   </si>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">room</t>
   </si>
   <si>
-    <t xml:space="preserve">out (devenir)</t>
+    <t xml:space="preserve">patient_died_during_stay</t>
   </si>
   <si>
     <t xml:space="preserve">Béatrice</t>
@@ -91,9 +91,6 @@
     <t xml:space="preserve">A01</t>
   </si>
   <si>
-    <t xml:space="preserve">out</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yves</t>
   </si>
   <si>
@@ -359,16 +356,27 @@
   </si>
   <si>
     <t xml:space="preserve">Z15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">François</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blache</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z19</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="168" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -473,7 +481,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -519,6 +527,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -766,6 +786,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="18.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="23.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="25.4"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -871,19 +892,17 @@
       <c r="K3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>22</v>
-      </c>
+      <c r="L3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>18865</v>
@@ -907,21 +926,19 @@
         <v>44713.4583333333</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="L4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>29165</v>
@@ -945,21 +962,19 @@
         <v>44755.4583333333</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="L5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>27</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>29452</v>
@@ -983,7 +998,7 @@
         <v>44698.4166666667</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -991,10 +1006,10 @@
         <v>33</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>33</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>30203</v>
@@ -1014,7 +1029,7 @@
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1022,10 +1037,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>23808</v>
@@ -1049,21 +1064,19 @@
         <v>44694.4166666667</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="L8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>29</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>39</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>31293</v>
@@ -1087,7 +1100,7 @@
         <v>44727.375</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1095,10 +1108,10 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>15472</v>
@@ -1122,21 +1135,19 @@
         <v>44708.5833333333</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="L10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>14</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>14591</v>
@@ -1160,21 +1171,19 @@
         <v>44700.4583333333</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="L11" s="1"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>36</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>47</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>48</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>20943</v>
@@ -1198,7 +1207,7 @@
         <v>44698.4583333333</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1206,10 +1215,10 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>19806</v>
@@ -1233,30 +1242,28 @@
         <v>44692.375</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="L13" s="1"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B14" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>19702</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>44685.4583333333</v>
@@ -1271,7 +1278,7 @@
         <v>44707.4166666667</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1279,10 +1286,10 @@
         <v>10</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>25135</v>
@@ -1306,21 +1313,19 @@
         <v>44695.4166666667</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="L15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>21046</v>
@@ -1344,21 +1349,19 @@
         <v>44711.4583333333</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="L16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>19702</v>
@@ -1382,7 +1385,7 @@
         <v>44707.4166666667</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1390,10 +1393,10 @@
         <v>1</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>54</v>
       </c>
       <c r="D18" s="9" t="n">
         <v>19702</v>
@@ -1417,7 +1420,7 @@
         <v>44707.4166666667</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1425,10 +1428,10 @@
         <v>6</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>19950</v>
@@ -1452,21 +1455,19 @@
         <v>44698.4166666667</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="L19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>21</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>69</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>32274</v>
@@ -1490,7 +1491,7 @@
         <v>44709.4583333333</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1498,10 +1499,10 @@
         <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>36884</v>
@@ -1521,7 +1522,7 @@
       </c>
       <c r="J21" s="4"/>
       <c r="K21" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1529,10 +1530,10 @@
         <v>15</v>
       </c>
       <c r="B22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>31242</v>
@@ -1556,21 +1557,19 @@
         <v>44734.5833333333</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="L22" s="1"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>24</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>33011</v>
@@ -1594,7 +1593,7 @@
         <v>44708.4166666667</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,10 +1601,10 @@
         <v>11</v>
       </c>
       <c r="B24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>31152</v>
@@ -1629,21 +1628,19 @@
         <v>44718.4166666667</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="L24" s="1"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
         <v>18</v>
       </c>
       <c r="B25" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>32558</v>
@@ -1667,21 +1664,19 @@
         <v>44699.7083333333</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="L25" s="1"/>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
         <v>37</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>30784</v>
@@ -1705,7 +1700,7 @@
         <v>44715.4583333333</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1713,10 +1708,10 @@
         <v>31</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>88</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>31607</v>
@@ -1740,7 +1735,7 @@
         <v>44710.4583333333</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1748,19 +1743,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>29452</v>
       </c>
       <c r="E28" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>89</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>44693</v>
@@ -1775,7 +1770,7 @@
         <v>44698.4166666667</v>
       </c>
       <c r="K28" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1783,10 +1778,10 @@
         <v>9</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>18208</v>
@@ -1810,21 +1805,19 @@
         <v>44706.4166666667</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L29" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="L29" s="1"/>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
         <v>34</v>
       </c>
       <c r="B30" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>36387</v>
@@ -1848,7 +1841,7 @@
         <v>44717.2916666667</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1856,19 +1849,19 @@
         <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>33011</v>
       </c>
       <c r="E31" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>44695.4166666667</v>
@@ -1883,7 +1876,7 @@
         <v>44708.4166666667</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1891,10 +1884,10 @@
         <v>16</v>
       </c>
       <c r="B32" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>26397</v>
@@ -1918,21 +1911,19 @@
         <v>44701.625</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="L32" s="1"/>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B33" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>54</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>19702</v>
@@ -1956,21 +1947,19 @@
         <v>44707.4166666667</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="L33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="n">
         <v>31</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>31607</v>
@@ -1994,7 +1983,7 @@
         <v>44710.4583333333</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,10 +1991,10 @@
         <v>7</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>28682</v>
@@ -2029,30 +2018,28 @@
         <v>44766.375</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>22</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="L35" s="1"/>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="n">
         <v>21</v>
       </c>
       <c r="B36" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>32274</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>44701.5833333333</v>
@@ -2067,7 +2054,7 @@
         <v>44709.4583333333</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2075,19 +2062,19 @@
         <v>37</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>30784</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>44703.7083333333</v>
@@ -2102,7 +2089,7 @@
         <v>44715.4583333333</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,19 +2097,19 @@
         <v>29</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>31293</v>
       </c>
       <c r="E38" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>44705.4166666667</v>
@@ -2137,7 +2124,7 @@
         <v>44727.375</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2145,19 +2132,19 @@
         <v>34</v>
       </c>
       <c r="B39" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C39" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>36387</v>
       </c>
       <c r="E39" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F39" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>98</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>44711.4583333333</v>
@@ -2172,7 +2159,45 @@
         <v>44717.2916666667</v>
       </c>
       <c r="K39" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="0" t="s">
         <v>111</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="D40" s="12" t="n">
+        <v>32955</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>44710.3125</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>44710.7291666667</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>44710.3125</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>44710.7291666667</v>
+      </c>
+      <c r="K40" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="L40" s="14" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2181,7 +2206,7 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:L39"/>
+  <autoFilter ref="A1:L40"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Add a stay before patient 38 died
</commit_message>
<xml_diff>
--- a/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
+++ b/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
@@ -11,7 +11,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$40</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$41</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="115">
   <si>
     <t xml:space="preserve">patient_ref</t>
   </si>
@@ -365,6 +365,9 @@
   </si>
   <si>
     <t xml:space="preserve">Z19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z20</t>
   </si>
 </sst>
 </file>
@@ -2176,16 +2179,16 @@
         <v>32955</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>44710.3125</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>44710.7291666667</v>
+        <v>44710.5625</v>
       </c>
       <c r="I40" s="4" t="n">
         <v>44710.3125</v>
@@ -2196,17 +2199,51 @@
       <c r="K40" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="L40" s="14" t="b">
+    </row>
+    <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" s="12" t="n">
+        <v>32955</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>44710.5625</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>44710.7291666667</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>44710.3125</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>44710.7291666667</v>
+      </c>
+      <c r="K41" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="L41" s="14" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:L40"/>
+  <autoFilter ref="A1:L41"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Add a stay with a sector
</commit_message>
<xml_diff>
--- a/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
+++ b/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
@@ -11,7 +11,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$41</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$M$41</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="122">
   <si>
     <t xml:space="preserve">patient_ref</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">hospitalization_out_time</t>
   </si>
   <si>
+    <t xml:space="preserve">sector</t>
+  </si>
+  <si>
     <t xml:space="preserve">room</t>
   </si>
   <si>
@@ -368,6 +371,24 @@
   </si>
   <si>
     <t xml:space="preserve">Z20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aymeric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dermato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dermatologie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dermat1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D01</t>
   </si>
 </sst>
 </file>
@@ -378,8 +399,8 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="mm/dd/yy"/>
-    <numFmt numFmtId="168" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yy"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -484,7 +505,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -506,6 +527,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -533,7 +558,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -541,7 +566,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -781,7 +806,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1048576"/>
+  <dimension ref="A1:M1048576"/>
   <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15"/>
@@ -789,7 +814,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="18.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="23.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="25.4"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="25.4"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -829,25 +855,28 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>36558</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>44655.4166666667</v>
@@ -857,8 +886,9 @@
         <v>44655.4166666667</v>
       </c>
       <c r="J2" s="4"/>
-      <c r="K2" s="5" t="s">
-        <v>16</v>
+      <c r="K2" s="4"/>
+      <c r="L2" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -866,19 +896,19 @@
         <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>30815</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>44675.375</v>
@@ -892,29 +922,32 @@
       <c r="J3" s="4" t="n">
         <v>44724.4166666667</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L3" s="1"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>18865</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>44675.4583333333</v>
@@ -928,29 +961,32 @@
       <c r="J4" s="4" t="n">
         <v>44713.4583333333</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="1"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M4" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>29165</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>44676.4166666667</v>
@@ -964,29 +1000,32 @@
       <c r="J5" s="4" t="n">
         <v>44755.4583333333</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="1"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M5" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>27</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="6" t="s">
         <v>29</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>30</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>29452</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>44678.4166666667</v>
@@ -1000,8 +1039,12 @@
       <c r="J6" s="4" t="n">
         <v>44698.4166666667</v>
       </c>
-      <c r="K6" s="5" t="s">
-        <v>30</v>
+      <c r="K6" s="4"/>
+      <c r="L6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="M6" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1009,19 +1052,19 @@
         <v>33</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="6" t="s">
         <v>32</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>33</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>30203</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>44680.4166666667</v>
@@ -1031,8 +1074,9 @@
         <v>44680.4166666667</v>
       </c>
       <c r="J7" s="4"/>
-      <c r="K7" s="5" t="s">
-        <v>33</v>
+      <c r="K7" s="4"/>
+      <c r="L7" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1040,19 +1084,19 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>23808</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>44681.375</v>
@@ -1066,29 +1110,32 @@
       <c r="J8" s="4" t="n">
         <v>44694.4166666667</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="L8" s="1"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M8" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>29</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="6" t="s">
         <v>38</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>39</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>31293</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>44682.4583333333</v>
@@ -1102,8 +1149,12 @@
       <c r="J9" s="4" t="n">
         <v>44727.375</v>
       </c>
-      <c r="K9" s="5" t="s">
-        <v>39</v>
+      <c r="K9" s="4"/>
+      <c r="L9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="M9" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1111,19 +1162,19 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>15472</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>44684.4166666667</v>
@@ -1137,29 +1188,32 @@
       <c r="J10" s="4" t="n">
         <v>44708.5833333333</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L10" s="1"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="M10" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>14</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>14591</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>44684.8333333333</v>
@@ -1173,29 +1227,32 @@
       <c r="J11" s="4" t="n">
         <v>44700.4583333333</v>
       </c>
-      <c r="K11" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L11" s="1"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="M11" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>36</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="6" t="s">
         <v>47</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>48</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>20943</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G12" s="4" t="n">
         <v>44685.375</v>
@@ -1209,8 +1266,12 @@
       <c r="J12" s="4" t="n">
         <v>44698.4583333333</v>
       </c>
-      <c r="K12" s="5" t="s">
-        <v>48</v>
+      <c r="K12" s="4"/>
+      <c r="L12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="M12" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1218,19 +1279,19 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>19806</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>44685.4166666667</v>
@@ -1244,29 +1305,32 @@
       <c r="J13" s="4" t="n">
         <v>44692.375</v>
       </c>
-      <c r="K13" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="L13" s="1"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="M13" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>19702</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>44685.4583333333</v>
@@ -1280,8 +1344,12 @@
       <c r="J14" s="4" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K14" s="5" t="s">
-        <v>56</v>
+      <c r="K14" s="4"/>
+      <c r="L14" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="M14" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1289,19 +1357,19 @@
         <v>10</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>25135</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>44685.4583333333</v>
@@ -1315,29 +1383,32 @@
       <c r="J15" s="4" t="n">
         <v>44695.4166666667</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="L15" s="1"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="M15" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>21046</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>44685.4583333333</v>
@@ -1351,29 +1422,32 @@
       <c r="J16" s="4" t="n">
         <v>44711.4583333333</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="L16" s="1"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="M16" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>19702</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>44685.7083333333</v>
@@ -1387,43 +1461,51 @@
       <c r="J17" s="4" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>63</v>
+      <c r="K17" s="4"/>
+      <c r="L17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="M17" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B18" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="8" t="s">
+      <c r="B18" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="C18" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D18" s="10" t="n">
         <v>19702</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F18" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="10" t="n">
+      <c r="F18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="11" t="n">
         <v>44686.6666666667</v>
       </c>
-      <c r="H18" s="10" t="n">
+      <c r="H18" s="11" t="n">
         <v>44696.4583333333</v>
       </c>
-      <c r="I18" s="10" t="n">
+      <c r="I18" s="11" t="n">
         <v>44685.4583333333</v>
       </c>
-      <c r="J18" s="10" t="n">
+      <c r="J18" s="11" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K18" s="7" t="s">
-        <v>27</v>
+      <c r="K18" s="11"/>
+      <c r="L18" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="M18" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1431,19 +1513,19 @@
         <v>6</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>19950</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>44688.4166666667</v>
@@ -1457,29 +1539,32 @@
       <c r="J19" s="4" t="n">
         <v>44698.4166666667</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L19" s="1"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="M19" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>21</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="6" t="s">
         <v>68</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>32274</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G20" s="4" t="n">
         <v>44688.4166666667</v>
@@ -1493,8 +1578,12 @@
       <c r="J20" s="4" t="n">
         <v>44709.4583333333</v>
       </c>
-      <c r="K20" s="5" t="s">
-        <v>69</v>
+      <c r="K20" s="4"/>
+      <c r="L20" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="M20" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1502,19 +1591,19 @@
         <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C21" s="6" t="s">
         <v>71</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>72</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>36884</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>44689.4583333333</v>
@@ -1524,8 +1613,9 @@
         <v>44689.4583333333</v>
       </c>
       <c r="J21" s="4"/>
-      <c r="K21" s="5" t="s">
-        <v>72</v>
+      <c r="K21" s="4"/>
+      <c r="L21" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1533,19 +1623,19 @@
         <v>15</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>31242</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>44690.4583333333</v>
@@ -1559,29 +1649,32 @@
       <c r="J22" s="4" t="n">
         <v>44734.5833333333</v>
       </c>
-      <c r="K22" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="L22" s="1"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="M22" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>24</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>33011</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>44692</v>
@@ -1595,8 +1688,12 @@
       <c r="J23" s="4" t="n">
         <v>44708.4166666667</v>
       </c>
-      <c r="K23" s="5" t="s">
-        <v>77</v>
+      <c r="K23" s="4"/>
+      <c r="L23" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="M23" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1604,19 +1701,19 @@
         <v>11</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>31152</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>44692.4166666667</v>
@@ -1630,29 +1727,32 @@
       <c r="J24" s="4" t="n">
         <v>44718.4166666667</v>
       </c>
-      <c r="K24" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="L24" s="1"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="M24" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
         <v>18</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>32558</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>44692.4583333333</v>
@@ -1666,29 +1766,32 @@
       <c r="J25" s="4" t="n">
         <v>44699.7083333333</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L25" s="1"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="M25" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
         <v>37</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>84</v>
+        <v>53</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>85</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>30784</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G26" s="4" t="n">
         <v>44692.7083333333</v>
@@ -1702,8 +1805,12 @@
       <c r="J26" s="4" t="n">
         <v>44715.4583333333</v>
       </c>
-      <c r="K26" s="5" t="s">
-        <v>85</v>
+      <c r="K26" s="4"/>
+      <c r="L26" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="M26" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1711,19 +1818,19 @@
         <v>31</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C27" s="6" t="s">
         <v>87</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>88</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>31607</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>44692.9166666667</v>
@@ -1737,8 +1844,12 @@
       <c r="J27" s="4" t="n">
         <v>44710.4583333333</v>
       </c>
-      <c r="K27" s="5" t="s">
-        <v>27</v>
+      <c r="K27" s="4"/>
+      <c r="L27" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="M27" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1746,19 +1857,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>29452</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G28" s="4" t="n">
         <v>44693</v>
@@ -1772,8 +1883,12 @@
       <c r="J28" s="4" t="n">
         <v>44698.4166666667</v>
       </c>
-      <c r="K28" s="5" t="s">
-        <v>90</v>
+      <c r="K28" s="4"/>
+      <c r="L28" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="M28" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1781,19 +1896,19 @@
         <v>9</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>18208</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>44694.4166666667</v>
@@ -1807,29 +1922,32 @@
       <c r="J29" s="4" t="n">
         <v>44706.4166666667</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="L29" s="1"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="M29" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
         <v>34</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>36387</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>44694.9583333333</v>
@@ -1843,28 +1961,32 @@
       <c r="J30" s="4" t="n">
         <v>44717.2916666667</v>
       </c>
-      <c r="K30" s="5" t="s">
-        <v>95</v>
+      <c r="K30" s="4"/>
+      <c r="L30" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="M30" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="n">
+      <c r="A31" s="12" t="n">
         <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>33011</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>44695.4166666667</v>
@@ -1878,8 +2000,12 @@
       <c r="J31" s="4" t="n">
         <v>44708.4166666667</v>
       </c>
-      <c r="K31" s="5" t="s">
-        <v>98</v>
+      <c r="K31" s="4"/>
+      <c r="L31" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="M31" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1887,19 +2013,19 @@
         <v>16</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>26397</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>44696.4166666667</v>
@@ -1913,29 +2039,32 @@
       <c r="J32" s="4" t="n">
         <v>44701.625</v>
       </c>
-      <c r="K32" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="L32" s="1"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="M32" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>19702</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>44696.4583333333</v>
@@ -1949,29 +2078,32 @@
       <c r="J33" s="4" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K33" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="L33" s="1"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M33" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="n">
         <v>31</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>31607</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G34" s="4" t="n">
         <v>44697.4583333333</v>
@@ -1985,8 +2117,12 @@
       <c r="J34" s="4" t="n">
         <v>44710.4583333333</v>
       </c>
-      <c r="K34" s="5" t="s">
-        <v>102</v>
+      <c r="K34" s="4"/>
+      <c r="L34" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M34" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1994,19 +2130,19 @@
         <v>7</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>28682</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>44699.4166666667</v>
@@ -2020,29 +2156,32 @@
       <c r="J35" s="4" t="n">
         <v>44766.375</v>
       </c>
-      <c r="K35" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="L35" s="1"/>
+      <c r="K35" s="4"/>
+      <c r="L35" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="M35" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="n">
         <v>21</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>32274</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G36" s="4" t="n">
         <v>44701.5833333333</v>
@@ -2056,8 +2195,12 @@
       <c r="J36" s="4" t="n">
         <v>44709.4583333333</v>
       </c>
-      <c r="K36" s="5" t="s">
-        <v>105</v>
+      <c r="K36" s="4"/>
+      <c r="L36" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="M36" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2065,19 +2208,19 @@
         <v>37</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>30784</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>44703.7083333333</v>
@@ -2091,8 +2234,12 @@
       <c r="J37" s="4" t="n">
         <v>44715.4583333333</v>
       </c>
-      <c r="K37" s="5" t="s">
-        <v>108</v>
+      <c r="K37" s="4"/>
+      <c r="L37" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="M37" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2100,19 +2247,19 @@
         <v>29</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>31293</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G38" s="4" t="n">
         <v>44705.4166666667</v>
@@ -2126,8 +2273,12 @@
       <c r="J38" s="4" t="n">
         <v>44727.375</v>
       </c>
-      <c r="K38" s="5" t="s">
-        <v>109</v>
+      <c r="K38" s="4"/>
+      <c r="L38" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="M38" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2135,19 +2286,19 @@
         <v>34</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>36387</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>44711.4583333333</v>
@@ -2161,8 +2312,12 @@
       <c r="J39" s="4" t="n">
         <v>44717.2916666667</v>
       </c>
-      <c r="K39" s="5" t="s">
-        <v>110</v>
+      <c r="K39" s="4"/>
+      <c r="L39" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="M39" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2170,19 +2325,19 @@
         <v>38</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="D40" s="12" t="n">
+        <v>113</v>
+      </c>
+      <c r="D40" s="13" t="n">
         <v>32955</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G40" s="4" t="n">
         <v>44710.3125</v>
@@ -2196,8 +2351,12 @@
       <c r="J40" s="4" t="n">
         <v>44710.7291666667</v>
       </c>
-      <c r="K40" s="13" t="s">
-        <v>113</v>
+      <c r="K40" s="4"/>
+      <c r="L40" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="M40" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2205,19 +2364,19 @@
         <v>38</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="D41" s="12" t="n">
+        <v>113</v>
+      </c>
+      <c r="D41" s="13" t="n">
         <v>32955</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>44710.5625</v>
@@ -2231,11 +2390,53 @@
       <c r="J41" s="4" t="n">
         <v>44710.7291666667</v>
       </c>
-      <c r="K41" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="L41" s="14" t="b">
+      <c r="K41" s="4"/>
+      <c r="L41" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="M41" s="15" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <v>29327</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>44675.40625</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>44676.8229166667</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>44675.40625</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>44676.8229166667</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="L42" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="M42" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2243,7 +2444,7 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:L41"/>
+  <autoFilter ref="A1:M41"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Add patient death and unit sector in parsing of FHIR XML file  (#115)
* Add importAnalysesDF and importStaysDF functions for data integration

* Add tests for ETLCtrl.importAnalysesDF and ETLCtrl.importStaysDF functions

* Refactor getAnalysesDataFrameFromXML to convert string values to enums for sample, request_type, and result

* rename

* Simplify time variable assignments in importStaysDF function

* Update docstring of importAnalysesDF and importStaysDF

* Add scenario for patient death during stay with detailed patient journey

* Add patient that died in eg. excel file

* Add a stay before patient 38 died

* Add deceased patient handling and admission details in FHIR XML conversion

* Add patient death status handling in stays DataFrame extraction

* Add patient_died_during_stay column to stays DataFrame for improved tracking

* Add a stay with a sector

* format excel file

* Add sector

* add sector

* add validation functions for location checks in FHIR XML
</commit_message>
<xml_diff>
--- a/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
+++ b/custom/demo/test/sample-input-data/accidental_discovery_and_epidemic/demo-stays SALIOU.XLSX
@@ -11,7 +11,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$L$39</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$M$41</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="122">
   <si>
     <t xml:space="preserve">patient_ref</t>
   </si>
@@ -55,10 +55,13 @@
     <t xml:space="preserve">hospitalization_out_time</t>
   </si>
   <si>
+    <t xml:space="preserve">sector</t>
+  </si>
+  <si>
     <t xml:space="preserve">room</t>
   </si>
   <si>
-    <t xml:space="preserve">out (devenir)</t>
+    <t xml:space="preserve">patient_died_during_stay</t>
   </si>
   <si>
     <t xml:space="preserve">Béatrice</t>
@@ -91,9 +94,6 @@
     <t xml:space="preserve">A01</t>
   </si>
   <si>
-    <t xml:space="preserve">out</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yves</t>
   </si>
   <si>
@@ -359,16 +359,48 @@
   </si>
   <si>
     <t xml:space="preserve">Z15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">François</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blache</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Z20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aymeric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dermato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dermatologie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dermat1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="168" formatCode="mm/dd/yy"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -473,7 +505,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -498,6 +530,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -519,6 +555,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -758,7 +806,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1048576"/>
+  <dimension ref="A1:M1048576"/>
   <sheetFormatPr defaultColWidth="11.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15"/>
@@ -766,6 +814,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="18.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="23.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="24.71"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="25.4"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -805,25 +855,28 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>36558</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>44655.4166666667</v>
@@ -833,8 +886,9 @@
         <v>44655.4166666667</v>
       </c>
       <c r="J2" s="4"/>
-      <c r="K2" s="5" t="s">
-        <v>16</v>
+      <c r="K2" s="4"/>
+      <c r="L2" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -842,19 +896,19 @@
         <v>5</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>30815</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>44675.375</v>
@@ -868,11 +922,12 @@
       <c r="J3" s="4" t="n">
         <v>44724.4166666667</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>21</v>
-      </c>
+      <c r="K3" s="4"/>
       <c r="L3" s="1" t="s">
         <v>22</v>
+      </c>
+      <c r="M3" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -889,10 +944,10 @@
         <v>18865</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>44675.4583333333</v>
@@ -906,11 +961,12 @@
       <c r="J4" s="4" t="n">
         <v>44713.4583333333</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="4"/>
+      <c r="L4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>22</v>
+      <c r="M4" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -927,10 +983,10 @@
         <v>29165</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>44676.4166666667</v>
@@ -944,11 +1000,12 @@
       <c r="J5" s="4" t="n">
         <v>44755.4583333333</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="4"/>
+      <c r="L5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="L5" s="1" t="s">
-        <v>22</v>
+      <c r="M5" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -958,17 +1015,17 @@
       <c r="B6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>30</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>29452</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>44678.4166666667</v>
@@ -982,8 +1039,12 @@
       <c r="J6" s="4" t="n">
         <v>44698.4166666667</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="4"/>
+      <c r="L6" s="5" t="s">
         <v>31</v>
+      </c>
+      <c r="M6" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -993,17 +1054,17 @@
       <c r="B7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>33</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>30203</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>44680.4166666667</v>
@@ -1013,7 +1074,8 @@
         <v>44680.4166666667</v>
       </c>
       <c r="J7" s="4"/>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="4"/>
+      <c r="L7" s="5" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1031,10 +1093,10 @@
         <v>23808</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>44681.375</v>
@@ -1048,11 +1110,12 @@
       <c r="J8" s="4" t="n">
         <v>44694.4166666667</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" s="4"/>
+      <c r="L8" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L8" s="1" t="s">
-        <v>22</v>
+      <c r="M8" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1062,17 +1125,17 @@
       <c r="B9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>39</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>31293</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>44682.4583333333</v>
@@ -1086,8 +1149,12 @@
       <c r="J9" s="4" t="n">
         <v>44727.375</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="4"/>
+      <c r="L9" s="5" t="s">
         <v>40</v>
+      </c>
+      <c r="M9" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1104,10 +1171,10 @@
         <v>15472</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>44684.4166666667</v>
@@ -1121,11 +1188,12 @@
       <c r="J10" s="4" t="n">
         <v>44708.5833333333</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="K10" s="4"/>
+      <c r="L10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L10" s="1" t="s">
-        <v>22</v>
+      <c r="M10" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1142,10 +1210,10 @@
         <v>14591</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>44684.8333333333</v>
@@ -1159,11 +1227,12 @@
       <c r="J11" s="4" t="n">
         <v>44700.4583333333</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="K11" s="4"/>
+      <c r="L11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="1" t="s">
-        <v>22</v>
+      <c r="M11" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1173,17 +1242,17 @@
       <c r="B12" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>48</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>20943</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G12" s="4" t="n">
         <v>44685.375</v>
@@ -1197,8 +1266,12 @@
       <c r="J12" s="4" t="n">
         <v>44698.4583333333</v>
       </c>
-      <c r="K12" s="5" t="s">
+      <c r="K12" s="4"/>
+      <c r="L12" s="5" t="s">
         <v>49</v>
+      </c>
+      <c r="M12" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1215,10 +1288,10 @@
         <v>19806</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>44685.4166666667</v>
@@ -1232,11 +1305,12 @@
       <c r="J13" s="4" t="n">
         <v>44692.375</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="K13" s="4"/>
+      <c r="L13" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="L13" s="1" t="s">
-        <v>22</v>
+      <c r="M13" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1270,8 +1344,12 @@
       <c r="J14" s="4" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="K14" s="4"/>
+      <c r="L14" s="5" t="s">
         <v>57</v>
+      </c>
+      <c r="M14" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1288,10 +1366,10 @@
         <v>25135</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>44685.4583333333</v>
@@ -1305,11 +1383,12 @@
       <c r="J15" s="4" t="n">
         <v>44695.4166666667</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="K15" s="4"/>
+      <c r="L15" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L15" s="1" t="s">
-        <v>22</v>
+      <c r="M15" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1326,10 +1405,10 @@
         <v>21046</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>44685.4583333333</v>
@@ -1343,11 +1422,12 @@
       <c r="J16" s="4" t="n">
         <v>44711.4583333333</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="K16" s="4"/>
+      <c r="L16" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="L16" s="1" t="s">
-        <v>22</v>
+      <c r="M16" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1364,10 +1444,10 @@
         <v>19702</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>44685.7083333333</v>
@@ -1381,43 +1461,51 @@
       <c r="J17" s="4" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="K17" s="4"/>
+      <c r="L17" s="1" t="s">
         <v>64</v>
       </c>
+      <c r="M17" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="10" t="n">
         <v>19702</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F18" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="10" t="n">
+      <c r="F18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="11" t="n">
         <v>44686.6666666667</v>
       </c>
-      <c r="H18" s="10" t="n">
+      <c r="H18" s="11" t="n">
         <v>44696.4583333333</v>
       </c>
-      <c r="I18" s="10" t="n">
+      <c r="I18" s="11" t="n">
         <v>44685.4583333333</v>
       </c>
-      <c r="J18" s="10" t="n">
+      <c r="J18" s="11" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="K18" s="11"/>
+      <c r="L18" s="8" t="s">
         <v>28</v>
+      </c>
+      <c r="M18" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1434,10 +1522,10 @@
         <v>19950</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>44688.4166666667</v>
@@ -1451,11 +1539,12 @@
       <c r="J19" s="4" t="n">
         <v>44698.4166666667</v>
       </c>
-      <c r="K19" s="1" t="s">
+      <c r="K19" s="4"/>
+      <c r="L19" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="L19" s="1" t="s">
-        <v>22</v>
+      <c r="M19" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1465,17 +1554,17 @@
       <c r="B20" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>69</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>32274</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G20" s="4" t="n">
         <v>44688.4166666667</v>
@@ -1489,8 +1578,12 @@
       <c r="J20" s="4" t="n">
         <v>44709.4583333333</v>
       </c>
-      <c r="K20" s="5" t="s">
+      <c r="K20" s="4"/>
+      <c r="L20" s="5" t="s">
         <v>70</v>
+      </c>
+      <c r="M20" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1500,17 +1593,17 @@
       <c r="B21" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>72</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>36884</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>44689.4583333333</v>
@@ -1520,7 +1613,8 @@
         <v>44689.4583333333</v>
       </c>
       <c r="J21" s="4"/>
-      <c r="K21" s="5" t="s">
+      <c r="K21" s="4"/>
+      <c r="L21" s="5" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1538,10 +1632,10 @@
         <v>31242</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G22" s="4" t="n">
         <v>44690.4583333333</v>
@@ -1555,11 +1649,12 @@
       <c r="J22" s="4" t="n">
         <v>44734.5833333333</v>
       </c>
-      <c r="K22" s="1" t="s">
+      <c r="K22" s="4"/>
+      <c r="L22" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="L22" s="1" t="s">
-        <v>22</v>
+      <c r="M22" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1576,10 +1671,10 @@
         <v>33011</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>44692</v>
@@ -1593,8 +1688,12 @@
       <c r="J23" s="4" t="n">
         <v>44708.4166666667</v>
       </c>
-      <c r="K23" s="5" t="s">
+      <c r="K23" s="4"/>
+      <c r="L23" s="5" t="s">
         <v>78</v>
+      </c>
+      <c r="M23" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1611,10 +1710,10 @@
         <v>31152</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G24" s="4" t="n">
         <v>44692.4166666667</v>
@@ -1628,11 +1727,12 @@
       <c r="J24" s="4" t="n">
         <v>44718.4166666667</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="K24" s="4"/>
+      <c r="L24" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L24" s="1" t="s">
-        <v>22</v>
+      <c r="M24" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1649,10 +1749,10 @@
         <v>32558</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>44692.4583333333</v>
@@ -1666,11 +1766,12 @@
       <c r="J25" s="4" t="n">
         <v>44699.7083333333</v>
       </c>
-      <c r="K25" s="1" t="s">
+      <c r="K25" s="4"/>
+      <c r="L25" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="L25" s="1" t="s">
-        <v>22</v>
+      <c r="M25" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1680,17 +1781,17 @@
       <c r="B26" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="7" t="s">
         <v>85</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>30784</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G26" s="4" t="n">
         <v>44692.7083333333</v>
@@ -1704,8 +1805,12 @@
       <c r="J26" s="4" t="n">
         <v>44715.4583333333</v>
       </c>
-      <c r="K26" s="5" t="s">
+      <c r="K26" s="4"/>
+      <c r="L26" s="5" t="s">
         <v>86</v>
+      </c>
+      <c r="M26" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1715,17 +1820,17 @@
       <c r="B27" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>88</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>31607</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>44692.9166666667</v>
@@ -1739,8 +1844,12 @@
       <c r="J27" s="4" t="n">
         <v>44710.4583333333</v>
       </c>
-      <c r="K27" s="5" t="s">
+      <c r="K27" s="4"/>
+      <c r="L27" s="5" t="s">
         <v>28</v>
+      </c>
+      <c r="M27" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,8 +1883,12 @@
       <c r="J28" s="4" t="n">
         <v>44698.4166666667</v>
       </c>
-      <c r="K28" s="5" t="s">
+      <c r="K28" s="4"/>
+      <c r="L28" s="5" t="s">
         <v>91</v>
+      </c>
+      <c r="M28" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1792,10 +1905,10 @@
         <v>18208</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>44694.4166666667</v>
@@ -1809,11 +1922,12 @@
       <c r="J29" s="4" t="n">
         <v>44706.4166666667</v>
       </c>
-      <c r="K29" s="1" t="s">
+      <c r="K29" s="4"/>
+      <c r="L29" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="L29" s="1" t="s">
-        <v>22</v>
+      <c r="M29" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1830,10 +1944,10 @@
         <v>36387</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>44694.9583333333</v>
@@ -1847,12 +1961,16 @@
       <c r="J30" s="4" t="n">
         <v>44717.2916666667</v>
       </c>
-      <c r="K30" s="5" t="s">
+      <c r="K30" s="4"/>
+      <c r="L30" s="5" t="s">
         <v>96</v>
       </c>
+      <c r="M30" s="6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="n">
+      <c r="A31" s="12" t="n">
         <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -1882,8 +2000,12 @@
       <c r="J31" s="4" t="n">
         <v>44708.4166666667</v>
       </c>
-      <c r="K31" s="5" t="s">
+      <c r="K31" s="4"/>
+      <c r="L31" s="5" t="s">
         <v>99</v>
+      </c>
+      <c r="M31" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1900,10 +2022,10 @@
         <v>26397</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G32" s="4" t="n">
         <v>44696.4166666667</v>
@@ -1917,11 +2039,12 @@
       <c r="J32" s="4" t="n">
         <v>44701.625</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="K32" s="4"/>
+      <c r="L32" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="L32" s="1" t="s">
-        <v>22</v>
+      <c r="M32" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1938,10 +2061,10 @@
         <v>19702</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>44696.4583333333</v>
@@ -1955,11 +2078,12 @@
       <c r="J33" s="4" t="n">
         <v>44707.4166666667</v>
       </c>
-      <c r="K33" s="1" t="s">
+      <c r="K33" s="4"/>
+      <c r="L33" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L33" s="1" t="s">
-        <v>22</v>
+      <c r="M33" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1976,10 +2100,10 @@
         <v>31607</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G34" s="4" t="n">
         <v>44697.4583333333</v>
@@ -1993,8 +2117,12 @@
       <c r="J34" s="4" t="n">
         <v>44710.4583333333</v>
       </c>
-      <c r="K34" s="5" t="s">
+      <c r="K34" s="4"/>
+      <c r="L34" s="5" t="s">
         <v>103</v>
+      </c>
+      <c r="M34" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2011,10 +2139,10 @@
         <v>28682</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>44699.4166666667</v>
@@ -2028,11 +2156,12 @@
       <c r="J35" s="4" t="n">
         <v>44766.375</v>
       </c>
-      <c r="K35" s="1" t="s">
+      <c r="K35" s="4"/>
+      <c r="L35" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="L35" s="1" t="s">
-        <v>22</v>
+      <c r="M35" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2066,8 +2195,12 @@
       <c r="J36" s="4" t="n">
         <v>44709.4583333333</v>
       </c>
-      <c r="K36" s="5" t="s">
+      <c r="K36" s="4"/>
+      <c r="L36" s="5" t="s">
         <v>106</v>
+      </c>
+      <c r="M36" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2101,8 +2234,12 @@
       <c r="J37" s="4" t="n">
         <v>44715.4583333333</v>
       </c>
-      <c r="K37" s="5" t="s">
+      <c r="K37" s="4"/>
+      <c r="L37" s="5" t="s">
         <v>109</v>
+      </c>
+      <c r="M37" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2136,8 +2273,12 @@
       <c r="J38" s="4" t="n">
         <v>44727.375</v>
       </c>
-      <c r="K38" s="5" t="s">
+      <c r="K38" s="4"/>
+      <c r="L38" s="5" t="s">
         <v>110</v>
+      </c>
+      <c r="M38" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2171,17 +2312,139 @@
       <c r="J39" s="4" t="n">
         <v>44717.2916666667</v>
       </c>
-      <c r="K39" s="5" t="s">
+      <c r="K39" s="4"/>
+      <c r="L39" s="5" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="M39" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <v>32955</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>44710.3125</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>44710.5625</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>44710.3125</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>44710.7291666667</v>
+      </c>
+      <c r="K40" s="4"/>
+      <c r="L40" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="M40" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="D41" s="13" t="n">
+        <v>32955</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>44710.5625</v>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>44710.7291666667</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>44710.3125</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>44710.7291666667</v>
+      </c>
+      <c r="K41" s="4"/>
+      <c r="L41" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="M41" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="D42" s="13" t="n">
+        <v>29327</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>44675.40625</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>44676.8229166667</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>44675.40625</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>44676.8229166667</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="L42" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="M42" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:L39"/>
+  <autoFilter ref="A1:M41"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>